<commit_message>
tracking update 18.05.2026 16:31
</commit_message>
<xml_diff>
--- a/files/UAE_006_ФПЗ_ПРЕДВАРИТЕЛЬНЫЙ_09.04.2026.xlsx
+++ b/files/UAE_006_ФПЗ_ПРЕДВАРИТЕЛЬНЫЙ_09.04.2026.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zinov\OneDrive\Desktop\РАБОЧАЯ\001 ИМПОРТ\001 containers\2026\001 UAE\UAE#6_STPARTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B1767D6-D066-4D49-A933-7D95145F2938}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{414654EF-DF73-4745-8280-DBB8E0FFF2AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ФПЗ_Э6" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" refMode="R1C1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="47">
   <si>
     <t xml:space="preserve">
 Артикул</t>
@@ -177,6 +177,9 @@
   <si>
     <t>проезд Батюнинский проезд 9 стр.1</t>
   </si>
+  <si>
+    <t>ИТОГО ФАКТ</t>
+  </si>
 </sst>
 </file>
 
@@ -203,58 +206,80 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Calibri Light"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color indexed="2"/>
       <name val="Calibri Light"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Calibri Light"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <name val="Calibri Light"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color indexed="2"/>
       <name val="Calibri Light"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
     <font>
       <sz val="12"/>
       <name val="Calibri Light"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FFC00000"/>
       <name val="Calibri Light"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri Light"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFC9211E"/>
       <name val="Calibri Light"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF00A933"/>
       <name val="Calibri Light"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
     <font>
       <b/>
@@ -499,9 +524,6 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="170" fontId="9" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyProtection="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
@@ -562,6 +584,9 @@
     </xf>
     <xf numFmtId="173" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="9" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -834,7 +859,7 @@
     <col min="19" max="20" width="17.5703125" style="7" customWidth="1"/>
     <col min="21" max="21" width="14.140625" style="7" customWidth="1"/>
     <col min="22" max="22" width="21.5703125" style="7" customWidth="1"/>
-    <col min="23" max="23" width="16" style="5" customWidth="1"/>
+    <col min="23" max="23" width="27.42578125" style="5" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="17.5703125" style="5" customWidth="1"/>
     <col min="25" max="25" width="19.140625" style="5" customWidth="1"/>
     <col min="26" max="26" width="34.42578125" style="5" customWidth="1"/>
@@ -1961,53 +1986,54 @@
       </c>
       <c r="M2" s="27">
         <f>L2+17/P2</f>
-        <v>4.4251898734177217</v>
+        <v>4.4294281780572167</v>
       </c>
       <c r="N2" s="27">
-        <f t="shared" ref="N2" si="1">M2*E2</f>
-        <v>1593.0683544303797</v>
+        <f>L2*E2</f>
+        <v>1515.6</v>
       </c>
       <c r="O2" s="28">
         <f>D2*E2*0.97</f>
         <v>349.2</v>
       </c>
       <c r="P2" s="24">
-        <v>79</v>
+        <f>21.1101082348139*3.67</f>
+        <v>77.474097221767011</v>
       </c>
       <c r="Q2" s="29">
-        <f t="shared" ref="Q2" si="2">M2*P2*1.0425</f>
-        <v>364.44757500000003</v>
+        <f>L2*P2</f>
+        <v>326.16594930363914</v>
       </c>
       <c r="R2" s="29">
-        <f t="shared" ref="R2:R7" si="3">$R$12/$N$10*N2</f>
-        <v>120333.669398741</v>
+        <f t="shared" ref="R2:R7" si="1">$R$12/$N$10*N2</f>
+        <v>117436.37507375304</v>
       </c>
       <c r="S2" s="29">
-        <f t="shared" ref="S2:S7" si="4">$S$12/$N$10*N2</f>
-        <v>33693.427431647484</v>
+        <f t="shared" ref="S2:S7" si="2">$S$12/$N$10*N2</f>
+        <v>32882.185020650853</v>
       </c>
       <c r="T2" s="29">
-        <f t="shared" ref="T2:T7" si="5">$T$12/$O$10*O2</f>
+        <f t="shared" ref="T2:T7" si="3">$T$12/$O$10*O2</f>
         <v>27069.917834702752</v>
       </c>
       <c r="U2" s="29">
-        <f t="shared" ref="U2:U7" si="6">$U$12/$O$10*O2</f>
+        <f t="shared" ref="U2:U7" si="4">$U$12/$O$10*O2</f>
         <v>1159.9806669888835</v>
       </c>
       <c r="V2" s="29">
-        <f t="shared" ref="V2" si="7">R2+S2+T2+U2</f>
-        <v>182256.99533208011</v>
+        <f t="shared" ref="V2" si="5">R2+S2+T2+U2</f>
+        <v>178548.45859609553</v>
       </c>
       <c r="W2" s="30">
-        <f t="shared" ref="W2" si="8">IFERROR(SUM(V2/E2),"")</f>
-        <v>506.26943147800034</v>
+        <f>Q2*($W$12/$R$12)</f>
+        <v>487.51604155042207</v>
       </c>
       <c r="X2" s="31">
         <v>510</v>
       </c>
       <c r="Y2" s="32">
         <f>IFERROR((X2-W2)/W2,"")</f>
-        <v>7.3687414053593067E-3</v>
+        <v>4.6119422815449014E-2</v>
       </c>
       <c r="Z2" s="33">
         <f>X2*E2</f>
@@ -2015,7 +2041,7 @@
       </c>
       <c r="AA2" s="33">
         <f>IFERROR(W2*E2,"")</f>
-        <v>182256.99533208011</v>
+        <v>175505.77495815195</v>
       </c>
       <c r="AB2" s="21"/>
       <c r="AC2" s="21"/>
@@ -3029,7 +3055,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="26">
-        <f t="shared" ref="E3:E7" si="9">SUM(F3:G3)</f>
+        <f t="shared" ref="E3:E7" si="6">SUM(F3:G3)</f>
         <v>17136</v>
       </c>
       <c r="F3" s="26">
@@ -3044,69 +3070,69 @@
         <v>25</v>
       </c>
       <c r="K3" s="26">
-        <f t="shared" ref="K3:K7" si="10">E3/J3</f>
+        <f t="shared" ref="K3:K7" si="7">E3/J3</f>
         <v>685.44</v>
       </c>
       <c r="L3" s="27">
         <v>5.0999999999999996</v>
       </c>
       <c r="M3" s="27">
-        <f t="shared" ref="M3:M7" si="11">L3+17/P3</f>
+        <f t="shared" ref="M3:M7" si="8">L3+17/P3</f>
         <v>5.3151898734177214</v>
       </c>
       <c r="N3" s="27">
-        <f t="shared" ref="N3:N7" si="12">M3*E3</f>
-        <v>91081.093670886068</v>
+        <f t="shared" ref="N3:N7" si="9">L3*E3</f>
+        <v>87393.599999999991</v>
       </c>
       <c r="O3" s="28">
-        <f t="shared" ref="O3:O7" si="13">D3*E3*0.97</f>
+        <f t="shared" ref="O3:O7" si="10">D3*E3*0.97</f>
         <v>16621.919999999998</v>
       </c>
       <c r="P3" s="24">
         <v>79</v>
       </c>
       <c r="Q3" s="29">
-        <f t="shared" ref="Q3:Q7" si="14">M3*P3*1.0425</f>
-        <v>437.74574999999999</v>
+        <f t="shared" ref="Q3:Q7" si="11">L3*P3</f>
+        <v>402.9</v>
       </c>
       <c r="R3" s="29">
+        <f t="shared" si="1"/>
+        <v>6771699.3854879541</v>
+      </c>
+      <c r="S3" s="29">
+        <f t="shared" si="2"/>
+        <v>1896075.8279366272</v>
+      </c>
+      <c r="T3" s="29">
         <f t="shared" si="3"/>
-        <v>6879881.9484347142</v>
-      </c>
-      <c r="S3" s="29">
+        <v>1288528.0889318509</v>
+      </c>
+      <c r="U3" s="29">
         <f t="shared" si="4"/>
-        <v>1926366.9455617203</v>
-      </c>
-      <c r="T3" s="29">
-        <f t="shared" si="5"/>
-        <v>1288528.0889318509</v>
-      </c>
-      <c r="U3" s="29">
-        <f t="shared" si="6"/>
         <v>55215.079748670847</v>
       </c>
       <c r="V3" s="29">
-        <f t="shared" ref="V3:V7" si="15">R3+S3+T3+U3</f>
-        <v>10149992.062676957</v>
+        <f t="shared" ref="V3:V7" si="12">R3+S3+T3+U3</f>
+        <v>10011518.382105105</v>
       </c>
       <c r="W3" s="30">
-        <f t="shared" ref="W3:W7" si="16">IFERROR(SUM(V3/E3),"")</f>
-        <v>592.3197982421193</v>
+        <f t="shared" ref="W3:W7" si="13">Q3*($W$12/$R$12)</f>
+        <v>602.20943835498497</v>
       </c>
       <c r="X3" s="31">
         <v>630</v>
       </c>
       <c r="Y3" s="32">
-        <f t="shared" ref="Y3:Y7" si="17">IFERROR((X3-W3)/W3,"")</f>
-        <v>6.3614624852499635E-2</v>
+        <f t="shared" ref="Y3:Y7" si="14">IFERROR((X3-W3)/W3,"")</f>
+        <v>4.6147668693019228E-2</v>
       </c>
       <c r="Z3" s="33">
         <f>X3*E3</f>
         <v>10795680</v>
       </c>
       <c r="AA3" s="33">
-        <f t="shared" ref="AA3:AA6" si="18">IFERROR(W3*E3,"")</f>
-        <v>10149992.062676957</v>
+        <f t="shared" ref="AA3:AA6" si="15">IFERROR(W3*E3,"")</f>
+        <v>10319460.935651023</v>
       </c>
       <c r="AB3" s="21"/>
       <c r="AC3" s="21"/>
@@ -4120,7 +4146,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="26">
-        <f t="shared" si="9"/>
+        <f t="shared" si="6"/>
         <v>5208</v>
       </c>
       <c r="F4" s="26">
@@ -4136,69 +4162,69 @@
         <v>26</v>
       </c>
       <c r="K4" s="26">
-        <f t="shared" si="10"/>
+        <f t="shared" si="7"/>
         <v>200.30769230769232</v>
       </c>
       <c r="L4" s="27">
         <v>6.8</v>
       </c>
       <c r="M4" s="27">
-        <f t="shared" si="11"/>
+        <f t="shared" si="8"/>
         <v>7.0151898734177216</v>
       </c>
       <c r="N4" s="27">
-        <f t="shared" si="12"/>
-        <v>36535.108860759494</v>
+        <f t="shared" si="9"/>
+        <v>35414.400000000001</v>
       </c>
       <c r="O4" s="28">
-        <f t="shared" si="13"/>
+        <f t="shared" si="10"/>
         <v>5051.76</v>
       </c>
       <c r="P4" s="24">
         <v>79</v>
       </c>
       <c r="Q4" s="29">
-        <f t="shared" si="14"/>
-        <v>577.75350000000003</v>
+        <f t="shared" si="11"/>
+        <v>537.19999999999993</v>
       </c>
       <c r="R4" s="29">
+        <f t="shared" si="1"/>
+        <v>2744087.3326813933</v>
+      </c>
+      <c r="S4" s="29">
+        <f t="shared" si="2"/>
+        <v>768344.45315079018</v>
+      </c>
+      <c r="T4" s="29">
         <f t="shared" si="3"/>
-        <v>2759708.1436405983</v>
-      </c>
-      <c r="S4" s="29">
+        <v>391611.47800869984</v>
+      </c>
+      <c r="U4" s="29">
         <f t="shared" si="4"/>
-        <v>772718.28021936759</v>
-      </c>
-      <c r="T4" s="29">
-        <f t="shared" si="5"/>
-        <v>391611.47800869984</v>
-      </c>
-      <c r="U4" s="29">
-        <f t="shared" si="6"/>
         <v>16781.053649105848</v>
       </c>
       <c r="V4" s="29">
-        <f t="shared" si="15"/>
-        <v>3940818.9555177717</v>
+        <f t="shared" si="12"/>
+        <v>3920824.3174899891</v>
       </c>
       <c r="W4" s="30">
-        <f t="shared" si="16"/>
-        <v>756.68566734212209</v>
+        <f t="shared" si="13"/>
+        <v>802.94591780664666</v>
       </c>
       <c r="X4" s="31">
         <v>820</v>
       </c>
       <c r="Y4" s="32">
-        <f t="shared" si="17"/>
-        <v>8.3673228383287793E-2</v>
+        <f t="shared" si="14"/>
+        <v>2.123939086699491E-2</v>
       </c>
       <c r="Z4" s="33">
-        <f t="shared" ref="Z4:Z6" si="19">X4*E4</f>
+        <f t="shared" ref="Z4:Z6" si="16">X4*E4</f>
         <v>4270560</v>
       </c>
       <c r="AA4" s="33">
-        <f t="shared" si="18"/>
-        <v>3940818.9555177717</v>
+        <f t="shared" si="15"/>
+        <v>4181742.3399370159</v>
       </c>
       <c r="AB4" s="21"/>
       <c r="AC4" s="21"/>
@@ -5212,7 +5238,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="26">
-        <f t="shared" si="9"/>
+        <f t="shared" si="6"/>
         <v>348</v>
       </c>
       <c r="F5" s="26">
@@ -5222,72 +5248,72 @@
       <c r="H5" s="26"/>
       <c r="I5" s="26"/>
       <c r="J5" s="26">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="K5" s="26">
-        <f t="shared" si="10"/>
-        <v>12.888888888888889</v>
+        <f t="shared" si="7"/>
+        <v>34.799999999999997</v>
       </c>
       <c r="L5" s="27">
         <v>9.6199999999999992</v>
       </c>
       <c r="M5" s="27">
-        <f t="shared" si="11"/>
+        <f t="shared" si="8"/>
         <v>9.8351898734177201</v>
       </c>
       <c r="N5" s="27">
-        <f t="shared" si="12"/>
-        <v>3422.6460759493666</v>
+        <f t="shared" si="9"/>
+        <v>3347.7599999999998</v>
       </c>
       <c r="O5" s="28">
-        <f t="shared" si="13"/>
+        <f t="shared" si="10"/>
         <v>337.56</v>
       </c>
       <c r="P5" s="24">
         <v>79</v>
       </c>
       <c r="Q5" s="29">
-        <f t="shared" si="14"/>
-        <v>810.00164999999993</v>
+        <f t="shared" si="11"/>
+        <v>759.9799999999999</v>
       </c>
       <c r="R5" s="29">
+        <f t="shared" si="1"/>
+        <v>259401.42452949818</v>
+      </c>
+      <c r="S5" s="29">
+        <f t="shared" si="2"/>
+        <v>72632.398868259494</v>
+      </c>
+      <c r="T5" s="29">
         <f t="shared" si="3"/>
-        <v>258532.25960254198</v>
-      </c>
-      <c r="S5" s="29">
+        <v>26167.587240212662</v>
+      </c>
+      <c r="U5" s="29">
         <f t="shared" si="4"/>
-        <v>72389.032688711755</v>
-      </c>
-      <c r="T5" s="29">
-        <f t="shared" si="5"/>
-        <v>26167.587240212662</v>
-      </c>
-      <c r="U5" s="29">
-        <f t="shared" si="6"/>
         <v>1121.3146447559207</v>
       </c>
       <c r="V5" s="29">
-        <f t="shared" si="15"/>
-        <v>358210.19417622231</v>
+        <f t="shared" si="12"/>
+        <v>359322.72528272623</v>
       </c>
       <c r="W5" s="30">
-        <f t="shared" si="16"/>
-        <v>1029.3396384374205</v>
+        <f t="shared" si="13"/>
+        <v>1135.9323131323442</v>
       </c>
       <c r="X5" s="31">
         <v>1160</v>
       </c>
       <c r="Y5" s="32">
-        <f t="shared" si="17"/>
-        <v>0.12693610221882376</v>
+        <f t="shared" si="14"/>
+        <v>2.118760650561026E-2</v>
       </c>
       <c r="Z5" s="33">
-        <f t="shared" si="19"/>
+        <f t="shared" si="16"/>
         <v>403680</v>
       </c>
       <c r="AA5" s="33">
-        <f t="shared" si="18"/>
-        <v>358210.19417622231</v>
+        <f t="shared" si="15"/>
+        <v>395304.44497005577</v>
       </c>
       <c r="AB5" s="21"/>
       <c r="AC5" s="21"/>
@@ -6301,7 +6327,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="26">
-        <f t="shared" si="9"/>
+        <f t="shared" si="6"/>
         <v>192</v>
       </c>
       <c r="F6" s="26">
@@ -6314,69 +6340,69 @@
         <v>29</v>
       </c>
       <c r="K6" s="26">
-        <f t="shared" si="10"/>
+        <f t="shared" si="7"/>
         <v>6.6206896551724137</v>
       </c>
       <c r="L6" s="27">
         <v>36.44</v>
       </c>
       <c r="M6" s="27">
-        <f t="shared" si="11"/>
+        <f t="shared" si="8"/>
         <v>36.655189873417719</v>
       </c>
       <c r="N6" s="27">
-        <f t="shared" si="12"/>
-        <v>7037.7964556962015</v>
+        <f t="shared" si="9"/>
+        <v>6996.48</v>
       </c>
       <c r="O6" s="28">
-        <f t="shared" si="13"/>
+        <f t="shared" si="10"/>
         <v>186.24</v>
       </c>
       <c r="P6" s="24">
         <v>79</v>
       </c>
       <c r="Q6" s="29">
-        <f t="shared" si="14"/>
-        <v>3018.8297999999995</v>
+        <f t="shared" si="11"/>
+        <v>2878.7599999999998</v>
       </c>
       <c r="R6" s="29">
+        <f t="shared" si="1"/>
+        <v>542122.75631829747</v>
+      </c>
+      <c r="S6" s="29">
+        <f t="shared" si="2"/>
+        <v>151794.3717691233</v>
+      </c>
+      <c r="T6" s="29">
         <f t="shared" si="3"/>
-        <v>531605.48299146339</v>
-      </c>
-      <c r="S6" s="29">
+        <v>14437.289511841469</v>
+      </c>
+      <c r="U6" s="29">
         <f t="shared" si="4"/>
-        <v>148849.53523760979</v>
-      </c>
-      <c r="T6" s="29">
-        <f t="shared" si="5"/>
-        <v>14437.289511841469</v>
-      </c>
-      <c r="U6" s="29">
-        <f t="shared" si="6"/>
         <v>618.6563557274045</v>
       </c>
       <c r="V6" s="29">
-        <f t="shared" si="15"/>
-        <v>695510.96409664198</v>
+        <f t="shared" si="12"/>
+        <v>708973.07395498955</v>
       </c>
       <c r="W6" s="30">
-        <f t="shared" si="16"/>
-        <v>3622.4529380033437</v>
+        <f t="shared" si="13"/>
+        <v>4302.845477187383</v>
       </c>
       <c r="X6" s="31">
         <v>4400</v>
       </c>
       <c r="Y6" s="32">
-        <f t="shared" si="17"/>
-        <v>0.21464656002549248</v>
+        <f t="shared" si="14"/>
+        <v>2.2579133582115853E-2</v>
       </c>
       <c r="Z6" s="33">
-        <f t="shared" si="19"/>
+        <f t="shared" si="16"/>
         <v>844800</v>
       </c>
       <c r="AA6" s="33">
-        <f t="shared" si="18"/>
-        <v>695510.96409664198</v>
+        <f t="shared" si="15"/>
+        <v>826146.33161997749</v>
       </c>
       <c r="AB6" s="21"/>
       <c r="AC6" s="21"/>
@@ -7390,7 +7416,7 @@
         <v>4</v>
       </c>
       <c r="E7" s="26">
-        <f t="shared" si="9"/>
+        <f t="shared" si="6"/>
         <v>396</v>
       </c>
       <c r="F7" s="26">
@@ -7403,61 +7429,61 @@
         <v>30</v>
       </c>
       <c r="K7" s="26">
-        <f t="shared" si="10"/>
+        <f t="shared" si="7"/>
         <v>13.2</v>
       </c>
       <c r="L7" s="27">
         <v>15.11</v>
       </c>
       <c r="M7" s="27">
-        <f t="shared" si="11"/>
+        <f t="shared" si="8"/>
         <v>15.32518987341772</v>
       </c>
       <c r="N7" s="27">
-        <f t="shared" si="12"/>
-        <v>6068.7751898734168</v>
+        <f t="shared" si="9"/>
+        <v>5983.5599999999995</v>
       </c>
       <c r="O7" s="28">
-        <f t="shared" si="13"/>
+        <f t="shared" si="10"/>
         <v>1536.48</v>
       </c>
       <c r="P7" s="24">
         <v>79</v>
       </c>
       <c r="Q7" s="29">
-        <f t="shared" si="14"/>
-        <v>1262.1443249999998</v>
+        <f t="shared" si="11"/>
+        <v>1193.69</v>
       </c>
       <c r="R7" s="29">
+        <f t="shared" si="1"/>
+        <v>463636.57722110429</v>
+      </c>
+      <c r="S7" s="29">
+        <f t="shared" si="2"/>
+        <v>129818.24162190921</v>
+      </c>
+      <c r="T7" s="29">
         <f t="shared" si="3"/>
-        <v>458409.7005772416</v>
-      </c>
-      <c r="S7" s="29">
+        <v>119107.63847269211</v>
+      </c>
+      <c r="U7" s="29">
         <f t="shared" si="4"/>
-        <v>128354.71616162767</v>
-      </c>
-      <c r="T7" s="29">
-        <f t="shared" si="5"/>
-        <v>119107.63847269211</v>
-      </c>
-      <c r="U7" s="29">
-        <f t="shared" si="6"/>
         <v>5103.9149347510875</v>
       </c>
       <c r="V7" s="29">
-        <f t="shared" si="15"/>
-        <v>710975.97014631249</v>
+        <f t="shared" si="12"/>
+        <v>717666.37225045671</v>
       </c>
       <c r="W7" s="30">
-        <f t="shared" si="16"/>
-        <v>1795.3938640058395</v>
+        <f t="shared" si="13"/>
+        <v>1784.1930614791813</v>
       </c>
       <c r="X7" s="31">
         <v>1820</v>
       </c>
       <c r="Y7" s="32">
-        <f t="shared" si="17"/>
-        <v>1.3705146534955762E-2</v>
+        <f t="shared" si="14"/>
+        <v>2.0068982047902941E-2</v>
       </c>
       <c r="Z7" s="33">
         <f>SUM(Z2:Z2)</f>
@@ -7465,83 +7491,83 @@
       </c>
       <c r="AA7" s="33">
         <f>SUM(AA2:AA2)</f>
-        <v>182256.99533208011</v>
+        <v>175505.77495815195</v>
       </c>
       <c r="AB7" s="21"/>
       <c r="AC7" s="21"/>
       <c r="AD7" s="21"/>
     </row>
     <row r="8" spans="1:1024" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="47"/>
-      <c r="B8" s="48"/>
-      <c r="C8" s="49"/>
-      <c r="D8" s="50"/>
-      <c r="E8" s="50"/>
-      <c r="F8" s="50"/>
-      <c r="G8" s="50"/>
-      <c r="H8" s="50"/>
-      <c r="I8" s="50"/>
-      <c r="J8" s="50"/>
-      <c r="K8" s="50"/>
-      <c r="L8" s="50"/>
-      <c r="M8" s="51"/>
-      <c r="N8" s="51"/>
-      <c r="O8" s="58"/>
-      <c r="P8" s="48"/>
-      <c r="Q8" s="52"/>
-      <c r="R8" s="52"/>
-      <c r="S8" s="52"/>
-      <c r="T8" s="52"/>
+      <c r="A8" s="46"/>
+      <c r="B8" s="47"/>
+      <c r="C8" s="48"/>
+      <c r="D8" s="49"/>
+      <c r="E8" s="49"/>
+      <c r="F8" s="49"/>
+      <c r="G8" s="49"/>
+      <c r="H8" s="49"/>
+      <c r="I8" s="49"/>
+      <c r="J8" s="49"/>
+      <c r="K8" s="49"/>
+      <c r="L8" s="49"/>
+      <c r="M8" s="50"/>
+      <c r="N8" s="50"/>
+      <c r="O8" s="57"/>
+      <c r="P8" s="47"/>
+      <c r="Q8" s="51"/>
+      <c r="R8" s="51"/>
+      <c r="S8" s="51"/>
+      <c r="T8" s="51"/>
       <c r="U8" s="34"/>
-      <c r="V8" s="52"/>
-      <c r="W8" s="53"/>
-      <c r="X8" s="58"/>
-      <c r="Y8" s="54"/>
-      <c r="Z8" s="55">
+      <c r="V8" s="51"/>
+      <c r="W8" s="52"/>
+      <c r="X8" s="57"/>
+      <c r="Y8" s="53"/>
+      <c r="Z8" s="54">
         <f>SUM(Z2:Z7)</f>
         <v>16681920</v>
       </c>
-      <c r="AA8" s="55">
+      <c r="AA8" s="54">
         <f>SUM(AA2:AA7)</f>
-        <v>15509046.167131754</v>
+        <v>16073665.602094378</v>
       </c>
       <c r="AB8" s="21"/>
       <c r="AC8" s="21"/>
       <c r="AD8" s="21"/>
     </row>
     <row r="9" spans="1:1024" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="47"/>
-      <c r="B9" s="48"/>
-      <c r="C9" s="49"/>
-      <c r="D9" s="50"/>
-      <c r="E9" s="50"/>
-      <c r="F9" s="50"/>
-      <c r="G9" s="50"/>
-      <c r="H9" s="50"/>
-      <c r="I9" s="50"/>
-      <c r="J9" s="50"/>
-      <c r="K9" s="50"/>
-      <c r="L9" s="50"/>
-      <c r="M9" s="51"/>
-      <c r="N9" s="51"/>
-      <c r="O9" s="58"/>
-      <c r="P9" s="48"/>
-      <c r="Q9" s="52"/>
-      <c r="R9" s="52"/>
-      <c r="S9" s="52"/>
-      <c r="T9" s="52"/>
+      <c r="A9" s="46"/>
+      <c r="B9" s="47"/>
+      <c r="C9" s="48"/>
+      <c r="D9" s="49"/>
+      <c r="E9" s="49"/>
+      <c r="F9" s="49"/>
+      <c r="G9" s="49"/>
+      <c r="H9" s="49"/>
+      <c r="I9" s="49"/>
+      <c r="J9" s="49"/>
+      <c r="K9" s="49"/>
+      <c r="L9" s="49"/>
+      <c r="M9" s="50"/>
+      <c r="N9" s="50"/>
+      <c r="O9" s="57"/>
+      <c r="P9" s="47"/>
+      <c r="Q9" s="51"/>
+      <c r="R9" s="51"/>
+      <c r="S9" s="51"/>
+      <c r="T9" s="51"/>
       <c r="U9" s="34"/>
-      <c r="V9" s="52"/>
-      <c r="W9" s="53"/>
-      <c r="X9" s="58"/>
-      <c r="Y9" s="54"/>
-      <c r="Z9" s="55">
+      <c r="V9" s="51"/>
+      <c r="W9" s="52"/>
+      <c r="X9" s="57"/>
+      <c r="Y9" s="53"/>
+      <c r="Z9" s="54">
         <f>Z8-I25</f>
         <v>13994880</v>
       </c>
-      <c r="AA9" s="55">
+      <c r="AA9" s="54">
         <f>AA8-H25</f>
-        <v>13007376.620708454</v>
+        <v>13472120.828400843</v>
       </c>
       <c r="AB9" s="21"/>
       <c r="AC9" s="21"/>
@@ -7563,26 +7589,26 @@
       <c r="J10" s="39"/>
       <c r="K10" s="38">
         <f>SUM(K2:K7)</f>
-        <v>933.45727085175383</v>
+        <v>955.36838196286487</v>
       </c>
       <c r="L10" s="38"/>
       <c r="M10" s="39"/>
-      <c r="N10" s="59">
+      <c r="N10" s="58">
         <f>SUMIF(N2:N7,"&lt;&gt;#ДЕЛ/0!")</f>
-        <v>145738.48860759492</v>
-      </c>
-      <c r="O10" s="60">
+        <v>140651.4</v>
+      </c>
+      <c r="O10" s="59">
         <f>SUM(O2:O7)</f>
         <v>24083.16</v>
       </c>
       <c r="Q10" s="7"/>
       <c r="R10" s="40">
         <f>SUMIF(R2:R7,"&lt;&gt;#ДЕЛ/0!")</f>
-        <v>11008471.2046453</v>
+        <v>10898383.851312</v>
       </c>
       <c r="S10" s="40">
         <f>SUMIF(S2:S7,"&lt;&gt;#ДЕЛ/0!")</f>
-        <v>3082371.9373006849</v>
+        <v>3051547.4783673603</v>
       </c>
       <c r="T10" s="40">
         <f>SUMIF(T2:T7,"&lt;&gt;#ДЕЛ/0!")</f>
@@ -7594,9 +7620,11 @@
       </c>
       <c r="V10" s="40">
         <f>SUMIF(V2:V7,"&lt;&gt;#ДЕЛ/0!")</f>
-        <v>16037765.141945986</v>
-      </c>
-      <c r="W10" s="41"/>
+        <v>15896853.329679362</v>
+      </c>
+      <c r="W10" s="64" t="s">
+        <v>46</v>
+      </c>
       <c r="X10" s="21"/>
       <c r="AA10" s="21"/>
       <c r="AB10" s="21"/>
@@ -7606,55 +7634,58 @@
       <c r="AMJ10" s="5"/>
     </row>
     <row r="11" spans="1:1024" ht="30" x14ac:dyDescent="0.25">
-      <c r="N11" s="56" t="s">
+      <c r="N11" s="55" t="s">
         <v>23</v>
       </c>
-      <c r="O11" s="57">
+      <c r="O11" s="56">
         <f>(O10/700)*20+O10</f>
         <v>24771.250285714286</v>
       </c>
       <c r="Q11" s="7"/>
-      <c r="R11" s="42" t="s">
+      <c r="R11" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="S11" s="42" t="s">
+      <c r="S11" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="T11" s="42" t="s">
+      <c r="T11" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="U11" s="42" t="s">
+      <c r="U11" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="V11" s="43"/>
-      <c r="Z11" s="61" t="s">
+      <c r="V11" s="42"/>
+      <c r="Z11" s="60" t="s">
         <v>25</v>
       </c>
-      <c r="AA11" s="62">
+      <c r="AA11" s="61">
         <f>(Z9-AA9)/AA9</f>
-        <v>7.5918719668606069E-2</v>
+        <v>3.8803034671209172E-2</v>
       </c>
     </row>
     <row r="12" spans="1:1024" ht="15.75" x14ac:dyDescent="0.25">
       <c r="N12" s="6"/>
       <c r="O12" s="6"/>
-      <c r="R12" s="44">
-        <v>11008471.2046453</v>
-      </c>
-      <c r="S12" s="44">
+      <c r="R12" s="43">
+        <v>10898383.851312</v>
+      </c>
+      <c r="S12" s="43">
         <f>R12*0.28</f>
-        <v>3082371.9373006844</v>
-      </c>
-      <c r="T12" s="45">
+        <v>3051547.4783673603</v>
+      </c>
+      <c r="T12" s="44">
         <f>915922+121000+650000+180000</f>
         <v>1866922</v>
       </c>
-      <c r="U12" s="45">
+      <c r="U12" s="44">
         <v>80000</v>
       </c>
-      <c r="V12" s="44">
+      <c r="V12" s="43">
         <f>R12+S12+T12+U12</f>
-        <v>16037765.141945984</v>
+        <v>15896853.329679361</v>
+      </c>
+      <c r="W12" s="43">
+        <v>16289673.909346335</v>
       </c>
     </row>
     <row r="13" spans="1:1024" x14ac:dyDescent="0.2">
@@ -7688,7 +7719,7 @@
       <c r="N16" s="6"/>
       <c r="O16" s="6"/>
       <c r="P16" s="5"/>
-      <c r="S16" s="46"/>
+      <c r="S16" s="45"/>
       <c r="T16" s="5"/>
       <c r="U16" s="5"/>
       <c r="V16" s="5"/>
@@ -7736,17 +7767,17 @@
       <c r="T22" s="5"/>
       <c r="U22" s="5"/>
       <c r="V22" s="5"/>
-      <c r="Z22" s="64">
+      <c r="Z22" s="63">
         <f>Z9-AA9</f>
-        <v>987503.3792915456</v>
+        <v>522759.17159915715</v>
       </c>
     </row>
     <row r="23" spans="8:26" x14ac:dyDescent="0.2">
-      <c r="H23" s="63">
+      <c r="H23" s="62">
         <f>G3*W3</f>
-        <v>1194116.7132561125</v>
-      </c>
-      <c r="I23" s="63">
+        <v>1214054.2277236497</v>
+      </c>
+      <c r="I23" s="62">
         <f>G3*X3</f>
         <v>1270080</v>
       </c>
@@ -7757,11 +7788,11 @@
       <c r="V23" s="5"/>
     </row>
     <row r="24" spans="8:26" x14ac:dyDescent="0.2">
-      <c r="H24" s="63">
+      <c r="H24" s="62">
         <f>G4*W4</f>
-        <v>1307552.8331671869</v>
-      </c>
-      <c r="I24" s="63">
+        <v>1387490.5459698855</v>
+      </c>
+      <c r="I24" s="62">
         <f>G4*X4</f>
         <v>1416960</v>
       </c>
@@ -7772,11 +7803,11 @@
       <c r="V24" s="5"/>
     </row>
     <row r="25" spans="8:26" x14ac:dyDescent="0.2">
-      <c r="H25" s="63">
+      <c r="H25" s="62">
         <f>SUM(H23:H24)</f>
-        <v>2501669.5464232992</v>
-      </c>
-      <c r="I25" s="63">
+        <v>2601544.7736935355</v>
+      </c>
+      <c r="I25" s="62">
         <f>SUM(I23:I24)</f>
         <v>2687040</v>
       </c>

</xml_diff>